<commit_message>
📊 Stock screener 2026-03-20
</commit_message>
<xml_diff>
--- a/output/stock_deviation_2026-03-20.xlsx
+++ b/output/stock_deviation_2026-03-20.xlsx
@@ -793,7 +793,7 @@
         <v>7.6</v>
       </c>
       <c r="U2" s="10" t="n">
-        <v>816.319</v>
+        <v>816.325</v>
       </c>
       <c r="V2" s="11" t="n">
         <v>6518</v>
@@ -5254,7 +5254,7 @@
         <v>16</v>
       </c>
       <c r="P57" s="7" t="n">
-        <v>25.44</v>
+        <v>25.51</v>
       </c>
       <c r="Q57" s="20" t="inlineStr">
         <is>
@@ -5265,7 +5265,7 @@
         <v>-3.8</v>
       </c>
       <c r="S57" s="21" t="n">
-        <v>-14.5</v>
+        <v>-14.2</v>
       </c>
       <c r="T57" s="9" t="n">
         <v>21.5</v>
@@ -34404,7 +34404,7 @@
       </c>
       <c r="O415" t="inlineStr"/>
       <c r="P415" s="7" t="n">
-        <v>9.199999999999999</v>
+        <v>6.9</v>
       </c>
       <c r="Q415" s="25" t="inlineStr">
         <is>
@@ -34412,10 +34412,10 @@
         </is>
       </c>
       <c r="R415" s="8" t="n">
-        <v>56.7</v>
+        <v>196.3</v>
       </c>
       <c r="S415" s="8" t="n">
-        <v>175.4</v>
+        <v>756</v>
       </c>
       <c r="T415" s="9" t="n">
         <v>3.8</v>
@@ -35136,7 +35136,7 @@
         <v>7.6</v>
       </c>
       <c r="U2" s="10" t="n">
-        <v>816.319</v>
+        <v>816.325</v>
       </c>
       <c r="V2" s="11" t="n">
         <v>6518</v>
@@ -55330,7 +55330,7 @@
         <v>16</v>
       </c>
       <c r="P6" s="7" t="n">
-        <v>25.44</v>
+        <v>25.51</v>
       </c>
       <c r="Q6" s="20" t="inlineStr">
         <is>
@@ -55341,7 +55341,7 @@
         <v>-3.8</v>
       </c>
       <c r="S6" s="21" t="n">
-        <v>-14.5</v>
+        <v>-14.2</v>
       </c>
       <c r="T6" s="9" t="n">
         <v>21.5</v>
@@ -64719,7 +64719,7 @@
       </c>
       <c r="O90" t="inlineStr"/>
       <c r="P90" s="7" t="n">
-        <v>9.199999999999999</v>
+        <v>6.9</v>
       </c>
       <c r="Q90" s="25" t="inlineStr">
         <is>
@@ -64727,10 +64727,10 @@
         </is>
       </c>
       <c r="R90" s="8" t="n">
-        <v>56.7</v>
+        <v>196.3</v>
       </c>
       <c r="S90" s="8" t="n">
-        <v>175.4</v>
+        <v>756</v>
       </c>
       <c r="T90" s="9" t="n">
         <v>3.8</v>
@@ -69932,7 +69932,7 @@
         <v>7.6</v>
       </c>
       <c r="U2" s="10" t="n">
-        <v>816.319</v>
+        <v>816.325</v>
       </c>
       <c r="V2" s="11" t="n">
         <v>6518</v>
@@ -74393,7 +74393,7 @@
         <v>16</v>
       </c>
       <c r="P57" s="7" t="n">
-        <v>25.44</v>
+        <v>25.51</v>
       </c>
       <c r="Q57" s="20" t="inlineStr">
         <is>
@@ -74404,7 +74404,7 @@
         <v>-3.8</v>
       </c>
       <c r="S57" s="21" t="n">
-        <v>-14.5</v>
+        <v>-14.2</v>
       </c>
       <c r="T57" s="9" t="n">
         <v>21.5</v>

</xml_diff>